<commit_message>
cap nhat file excel
</commit_message>
<xml_diff>
--- a/test-report/test_data.xlsx
+++ b/test-report/test_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BTL-AI\-Student-Performance-Prediction-Classification-\test-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CB16884-0BAE-415E-AC06-95A56FA8489E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4840AA-FAE1-415D-A5F9-0DD1EBCD8CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="58">
   <si>
     <t>TestID</t>
   </si>
@@ -170,16 +170,49 @@
   </si>
   <si>
     <t>≈92</t>
+  </si>
+  <si>
+    <t>Actual Output</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Check manually</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Running Total</t>
+  </si>
+  <si>
+    <t>Count</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -205,13 +238,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -225,9 +263,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{360A059E-2240-456E-9587-082F21D5AB66}" name="Table1" displayName="Table1" ref="A1:L13" totalsRowShown="0">
-  <autoFilter ref="A1:L13" xr:uid="{360A059E-2240-456E-9587-082F21D5AB66}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{360A059E-2240-456E-9587-082F21D5AB66}" name="Table1" displayName="Table1" ref="A1:N13" totalsRowShown="0">
+  <autoFilter ref="A1:N13" xr:uid="{360A059E-2240-456E-9587-082F21D5AB66}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{6E00A880-A64F-4F9A-8DB8-096530E8E90E}" name="TestID"/>
     <tableColumn id="2" xr3:uid="{BFF6B074-197D-400D-BDCD-9B9F1D18E1DF}" name="Description"/>
     <tableColumn id="3" xr3:uid="{BE02128B-266C-42D2-A71B-92F8E5D3D0E2}" name="Gender"/>
@@ -240,6 +278,8 @@
     <tableColumn id="10" xr3:uid="{8D3CFAD6-267C-47CC-95BC-C5AFA5B1CF0F}" name="Study_Attendance_Score"/>
     <tableColumn id="11" xr3:uid="{007A6FC7-C248-41AE-B790-294FDFCA7AE9}" name="Study_per_Activity"/>
     <tableColumn id="12" xr3:uid="{8A4CF740-01F3-4043-A084-73EAA322CDDB}" name="Expected Output"/>
+    <tableColumn id="13" xr3:uid="{9F82541C-3E22-4A14-8DD4-DDB6266C25C2}" name="Actual Output" dataDxfId="0"/>
+    <tableColumn id="14" xr3:uid="{EAFAB751-263A-42F7-A873-178434091E8E}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -530,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
@@ -545,9 +585,11 @@
     <col min="10" max="10" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -584,8 +626,14 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M1" t="s">
+        <v>50</v>
+      </c>
+      <c r="N1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -622,8 +670,14 @@
       <c r="L2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M2" s="1">
+        <v>79.841628232681401</v>
+      </c>
+      <c r="N2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -660,8 +714,14 @@
       <c r="L3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3" s="1">
+        <v>80.325178470080303</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -698,8 +758,14 @@
       <c r="L4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4" s="1">
+        <v>79.834268956959804</v>
+      </c>
+      <c r="N4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -736,8 +802,14 @@
       <c r="L5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5" s="1">
+        <v>80.178905472534694</v>
+      </c>
+      <c r="N5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -774,8 +846,14 @@
       <c r="L6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6" s="1">
+        <v>79.930335971105393</v>
+      </c>
+      <c r="N6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -812,8 +890,14 @@
       <c r="L7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M7" s="1">
+        <v>81.626234661657605</v>
+      </c>
+      <c r="N7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -850,8 +934,14 @@
       <c r="L8" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M8" s="1">
+        <v>78.857684974795902</v>
+      </c>
+      <c r="N8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -888,8 +978,14 @@
       <c r="L9" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M9" s="1">
+        <v>80.119694999608598</v>
+      </c>
+      <c r="N9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -926,8 +1022,14 @@
       <c r="L10" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M10" s="1">
+        <v>79.361410362711595</v>
+      </c>
+      <c r="N10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -964,8 +1066,14 @@
       <c r="L11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M11" s="1">
+        <v>80.295471398540997</v>
+      </c>
+      <c r="N11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1002,8 +1110,14 @@
       <c r="L12" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M12" s="1">
+        <v>79.943693807187003</v>
+      </c>
+      <c r="N12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1040,8 +1154,15 @@
       <c r="L13" t="s">
         <v>49</v>
       </c>
+      <c r="M13" s="1">
+        <v>80.028431660465898</v>
+      </c>
+      <c r="N13" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>